<commit_message>
Work done on Collections and workzone fields to display and edit
</commit_message>
<xml_diff>
--- a/documents/Account upload.xlsx
+++ b/documents/Account upload.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/darryllrobinson/Documents/projects/ciab/documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E69DEA63-A376-2D4B-9A5A-1AF663E22B21}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98EC56B4-9FE4-C149-B1CF-A3AE5E4F4C3B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="460" windowWidth="28380" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Account" sheetId="11" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Account!$B$1:$S$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Account!$B$1:$T$49</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="153">
   <si>
     <t>3RD101</t>
   </si>
@@ -492,6 +492,9 @@
   </si>
   <si>
     <t>Overdue</t>
+  </si>
+  <si>
+    <t>CustomerRefNo</t>
   </si>
 </sst>
 </file>
@@ -849,87 +852,91 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AC8A94F-0D88-45B1-B60B-5C961E12494A}">
-  <dimension ref="A1:S51"/>
+  <dimension ref="A1:T51"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="47.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.5" style="5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.1640625" style="5" bestFit="1" customWidth="1"/>
-    <col min="9" max="11" width="6.6640625" style="5" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="7.83203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.5" style="8" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="4" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="11.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="25.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="20" max="16384" width="8.83203125" style="1"/>
+    <col min="3" max="3" width="13" style="1" customWidth="1"/>
+    <col min="4" max="4" width="47.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.83203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.5" style="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.1640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="10" max="12" width="6.6640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="13" max="15" width="7.83203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.5" style="8" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="4" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="25.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="13">
+    <row r="1" spans="1:20" ht="13">
       <c r="A1" s="1" t="s">
         <v>137</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="M1" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="O1" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="O1" s="5" t="s">
+      <c r="P1" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="S1" s="9" t="s">
+      <c r="T1" s="9" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="2" spans="1:19" ht="13">
+    <row r="2" spans="1:20" ht="13">
       <c r="A2" s="1" t="s">
         <v>138</v>
       </c>
@@ -937,24 +944,27 @@
         <v>0</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="E2" s="1">
+      <c r="F2" s="1">
         <v>7</v>
       </c>
-      <c r="H2" s="6"/>
-      <c r="O2" s="5"/>
-      <c r="P2" s="1" t="s">
-        <v>99</v>
-      </c>
+      <c r="I2" s="6"/>
+      <c r="P2" s="5"/>
       <c r="Q2" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="S2" s="1" t="s">
+      <c r="R2" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="T2" s="1" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="3" spans="1:19" ht="13">
+    <row r="3" spans="1:20" ht="13">
       <c r="A3" s="1" t="s">
         <v>138</v>
       </c>
@@ -962,23 +972,26 @@
         <v>1</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="E3" s="1">
+      <c r="F3" s="1">
         <v>7</v>
       </c>
-      <c r="O3" s="5"/>
-      <c r="P3" s="1" t="s">
-        <v>99</v>
-      </c>
+      <c r="P3" s="5"/>
       <c r="Q3" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="S3" s="1" t="s">
+      <c r="R3" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="T3" s="1" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="4" spans="1:19" ht="13">
+    <row r="4" spans="1:20" ht="13">
       <c r="A4" s="1" t="s">
         <v>138</v>
       </c>
@@ -986,19 +999,22 @@
         <v>2</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="G4" s="5">
+      <c r="H4" s="5">
         <v>16915.78</v>
       </c>
-      <c r="O4" s="5">
+      <c r="P4" s="5">
         <v>16915.78</v>
       </c>
-      <c r="S4" s="1" t="s">
+      <c r="T4" s="1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="5" spans="1:19" ht="13">
+    <row r="5" spans="1:20" ht="13">
       <c r="A5" s="1" t="s">
         <v>138</v>
       </c>
@@ -1006,35 +1022,38 @@
         <v>3</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="E5" s="1">
-        <v>30</v>
-      </c>
-      <c r="G5" s="5">
+      <c r="F5" s="1">
+        <v>30</v>
+      </c>
+      <c r="H5" s="5">
         <v>29934.84</v>
       </c>
-      <c r="H5" s="6"/>
-      <c r="L5" s="7"/>
+      <c r="I5" s="6"/>
       <c r="M5" s="7"/>
       <c r="N5" s="7"/>
-      <c r="O5" s="5">
+      <c r="O5" s="7"/>
+      <c r="P5" s="5">
         <v>29934.84</v>
       </c>
-      <c r="P5" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="Q5" s="1" t="s">
         <v>97</v>
       </c>
       <c r="R5" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="S5" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="S5" s="1" t="s">
+      <c r="T5" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="6" spans="1:19" ht="13">
+    <row r="6" spans="1:20" ht="13">
       <c r="A6" s="1" t="s">
         <v>138</v>
       </c>
@@ -1042,31 +1061,34 @@
         <v>4</v>
       </c>
       <c r="C6" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="E6" s="1">
-        <v>30</v>
-      </c>
-      <c r="G6" s="5">
+      <c r="F6" s="1">
+        <v>30</v>
+      </c>
+      <c r="H6" s="5">
         <v>34658.080000000002</v>
       </c>
-      <c r="O6" s="5">
+      <c r="P6" s="5">
         <v>34658.080000000002</v>
       </c>
-      <c r="P6" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="Q6" s="1" t="s">
         <v>97</v>
       </c>
       <c r="R6" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="S6" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="S6" s="1" t="s">
+      <c r="T6" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="7" spans="1:19" ht="13">
+    <row r="7" spans="1:20" ht="13">
       <c r="A7" s="1" t="s">
         <v>138</v>
       </c>
@@ -1074,28 +1096,31 @@
         <v>5</v>
       </c>
       <c r="C7" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="E7" s="1">
-        <v>30</v>
-      </c>
-      <c r="G7" s="5">
+      <c r="F7" s="1">
+        <v>30</v>
+      </c>
+      <c r="H7" s="5">
         <v>8889.5</v>
       </c>
-      <c r="O7" s="5">
+      <c r="P7" s="5">
         <v>8889.5</v>
       </c>
-      <c r="P7" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="Q7" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="S7" s="1" t="s">
+      <c r="R7" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="T7" s="1" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="8" spans="1:19" ht="13">
+    <row r="8" spans="1:20" ht="13">
       <c r="A8" s="1" t="s">
         <v>138</v>
       </c>
@@ -1103,29 +1128,32 @@
         <v>6</v>
       </c>
       <c r="C8" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D8" s="2"/>
-      <c r="E8" s="1">
+      <c r="E8" s="2"/>
+      <c r="F8" s="1">
         <v>0</v>
       </c>
-      <c r="G8" s="5">
+      <c r="H8" s="5">
         <v>5000.01</v>
       </c>
-      <c r="O8" s="5">
+      <c r="P8" s="5">
         <v>5000.01</v>
-      </c>
-      <c r="P8" s="1" t="s">
-        <v>106</v>
       </c>
       <c r="Q8" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="S8" s="1" t="s">
+      <c r="R8" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="T8" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="9" spans="1:19" ht="13">
+    <row r="9" spans="1:20" ht="13">
       <c r="A9" s="1" t="s">
         <v>138</v>
       </c>
@@ -1133,31 +1161,34 @@
         <v>7</v>
       </c>
       <c r="C9" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E9" s="1">
-        <v>30</v>
-      </c>
-      <c r="G9" s="5">
+      <c r="F9" s="1">
+        <v>30</v>
+      </c>
+      <c r="H9" s="5">
         <v>23913.85</v>
       </c>
-      <c r="O9" s="5">
+      <c r="P9" s="5">
         <v>23913.85</v>
       </c>
-      <c r="P9" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="Q9" s="1" t="s">
         <v>97</v>
       </c>
       <c r="R9" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="S9" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="S9" s="1" t="s">
+      <c r="T9" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="10" spans="1:19" ht="13">
+    <row r="10" spans="1:20" ht="13">
       <c r="A10" s="1" t="s">
         <v>138</v>
       </c>
@@ -1165,29 +1196,32 @@
         <v>8</v>
       </c>
       <c r="C10" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="E10" s="1">
-        <v>30</v>
-      </c>
-      <c r="G10" s="5">
+      <c r="F10" s="1">
+        <v>30</v>
+      </c>
+      <c r="H10" s="5">
         <v>14947.7</v>
       </c>
-      <c r="H10" s="6"/>
-      <c r="O10" s="5">
+      <c r="I10" s="6"/>
+      <c r="P10" s="5">
         <v>14947.7</v>
       </c>
-      <c r="P10" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="Q10" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="S10" s="1" t="s">
+      <c r="R10" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="T10" s="1" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="11" spans="1:19" ht="13">
+    <row r="11" spans="1:20" ht="13">
       <c r="A11" s="1" t="s">
         <v>138</v>
       </c>
@@ -1195,31 +1229,34 @@
         <v>9</v>
       </c>
       <c r="C11" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="E11" s="1">
-        <v>30</v>
-      </c>
-      <c r="G11" s="5">
+      <c r="F11" s="1">
+        <v>30</v>
+      </c>
+      <c r="H11" s="5">
         <v>8746.2800000000007</v>
       </c>
-      <c r="O11" s="5">
+      <c r="P11" s="5">
         <v>8746.2800000000007</v>
       </c>
-      <c r="P11" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="Q11" s="1" t="s">
         <v>97</v>
       </c>
       <c r="R11" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="S11" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="S11" s="1" t="s">
+      <c r="T11" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="12" spans="1:19" ht="13">
+    <row r="12" spans="1:20" ht="13">
       <c r="A12" s="1" t="s">
         <v>138</v>
       </c>
@@ -1227,19 +1264,22 @@
         <v>10</v>
       </c>
       <c r="C12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="G12" s="5">
+      <c r="H12" s="5">
         <v>87175.63</v>
       </c>
-      <c r="O12" s="5">
+      <c r="P12" s="5">
         <v>87175.63</v>
       </c>
-      <c r="S12" s="1" t="s">
+      <c r="T12" s="1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="13" spans="1:19" ht="13">
+    <row r="13" spans="1:20" ht="13">
       <c r="A13" s="1" t="s">
         <v>138</v>
       </c>
@@ -1247,29 +1287,32 @@
         <v>11</v>
       </c>
       <c r="C13" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D13" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="D13" s="2"/>
-      <c r="E13" s="1">
+      <c r="E13" s="2"/>
+      <c r="F13" s="1">
         <v>0</v>
       </c>
-      <c r="G13" s="5">
+      <c r="H13" s="5">
         <v>5694.43</v>
       </c>
-      <c r="O13" s="5">
+      <c r="P13" s="5">
         <v>5694.43</v>
-      </c>
-      <c r="P13" s="1" t="s">
-        <v>106</v>
       </c>
       <c r="Q13" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="S13" s="1" t="s">
+      <c r="R13" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="T13" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="14" spans="1:19" ht="13">
+    <row r="14" spans="1:20" ht="13">
       <c r="A14" s="1" t="s">
         <v>138</v>
       </c>
@@ -1277,29 +1320,32 @@
         <v>12</v>
       </c>
       <c r="C14" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D14" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="E14" s="1">
-        <v>30</v>
-      </c>
-      <c r="G14" s="5">
+      <c r="F14" s="1">
+        <v>30</v>
+      </c>
+      <c r="H14" s="5">
         <v>5100</v>
       </c>
-      <c r="H14" s="6"/>
-      <c r="O14" s="5">
+      <c r="I14" s="6"/>
+      <c r="P14" s="5">
         <v>5100</v>
       </c>
-      <c r="P14" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="Q14" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="S14" s="1" t="s">
+      <c r="R14" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="T14" s="1" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="15" spans="1:19" ht="13">
+    <row r="15" spans="1:20" ht="13">
       <c r="A15" s="1" t="s">
         <v>138</v>
       </c>
@@ -1307,29 +1353,32 @@
         <v>13</v>
       </c>
       <c r="C15" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E15" s="1">
-        <v>30</v>
-      </c>
-      <c r="G15" s="5">
+      <c r="F15" s="1">
+        <v>30</v>
+      </c>
+      <c r="H15" s="5">
         <v>7343.87</v>
       </c>
-      <c r="H15" s="6"/>
-      <c r="O15" s="5">
+      <c r="I15" s="6"/>
+      <c r="P15" s="5">
         <v>7343.87</v>
       </c>
-      <c r="P15" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="Q15" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="S15" s="1" t="s">
+      <c r="R15" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="T15" s="1" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="16" spans="1:19" ht="13">
+    <row r="16" spans="1:20" ht="13">
       <c r="A16" s="1" t="s">
         <v>138</v>
       </c>
@@ -1337,28 +1386,31 @@
         <v>14</v>
       </c>
       <c r="C16" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="E16" s="1">
-        <v>30</v>
-      </c>
-      <c r="G16" s="5">
+      <c r="F16" s="1">
+        <v>30</v>
+      </c>
+      <c r="H16" s="5">
         <v>32478.880000000001</v>
       </c>
-      <c r="O16" s="5">
+      <c r="P16" s="5">
         <v>32478.880000000001</v>
       </c>
-      <c r="P16" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="Q16" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="S16" s="1" t="s">
+      <c r="R16" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="T16" s="1" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="17" spans="1:19" ht="13">
+    <row r="17" spans="1:20" ht="13">
       <c r="A17" s="1" t="s">
         <v>138</v>
       </c>
@@ -1366,28 +1418,31 @@
         <v>15</v>
       </c>
       <c r="C17" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D17" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="E17" s="1">
-        <v>30</v>
-      </c>
-      <c r="G17" s="5">
+      <c r="F17" s="1">
+        <v>30</v>
+      </c>
+      <c r="H17" s="5">
         <v>4325.84</v>
       </c>
-      <c r="O17" s="5">
+      <c r="P17" s="5">
         <v>4325.84</v>
       </c>
-      <c r="P17" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="Q17" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="S17" s="1" t="s">
+      <c r="R17" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="T17" s="1" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="18" spans="1:19" ht="13">
+    <row r="18" spans="1:20" ht="13">
       <c r="A18" s="1" t="s">
         <v>138</v>
       </c>
@@ -1395,29 +1450,32 @@
         <v>16</v>
       </c>
       <c r="C18" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D18" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="D18" s="4"/>
-      <c r="E18" s="1">
-        <v>30</v>
-      </c>
-      <c r="G18" s="5">
+      <c r="E18" s="4"/>
+      <c r="F18" s="1">
+        <v>30</v>
+      </c>
+      <c r="H18" s="5">
         <v>19108.419999999998</v>
       </c>
-      <c r="O18" s="5">
+      <c r="P18" s="5">
         <v>19108.419999999998</v>
       </c>
-      <c r="P18" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="Q18" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="S18" s="1" t="s">
+      <c r="R18" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="T18" s="1" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="19" spans="1:19" ht="13">
+    <row r="19" spans="1:20" ht="13">
       <c r="A19" s="1" t="s">
         <v>138</v>
       </c>
@@ -1425,34 +1483,37 @@
         <v>17</v>
       </c>
       <c r="C19" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D19" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="E19" s="1">
+      <c r="F19" s="1">
         <v>0</v>
       </c>
-      <c r="G19" s="5">
+      <c r="H19" s="5">
         <v>12075.93</v>
       </c>
-      <c r="L19" s="7"/>
       <c r="M19" s="7"/>
       <c r="N19" s="7"/>
-      <c r="O19" s="5">
+      <c r="O19" s="7"/>
+      <c r="P19" s="5">
         <v>12075.93</v>
-      </c>
-      <c r="P19" s="1" t="s">
-        <v>104</v>
       </c>
       <c r="Q19" s="1" t="s">
         <v>104</v>
       </c>
       <c r="R19" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="S19" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="S19" s="1" t="s">
+      <c r="T19" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="20" spans="1:19" ht="13">
+    <row r="20" spans="1:20" ht="13">
       <c r="A20" s="1" t="s">
         <v>138</v>
       </c>
@@ -1460,32 +1521,35 @@
         <v>18</v>
       </c>
       <c r="C20" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D20" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="D20" s="2"/>
-      <c r="E20" s="1">
-        <v>30</v>
-      </c>
-      <c r="G20" s="5">
+      <c r="E20" s="2"/>
+      <c r="F20" s="1">
+        <v>30</v>
+      </c>
+      <c r="H20" s="5">
         <v>29895.4</v>
       </c>
-      <c r="O20" s="5">
+      <c r="P20" s="5">
         <v>29895.4</v>
       </c>
-      <c r="P20" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="Q20" s="1" t="s">
         <v>97</v>
       </c>
       <c r="R20" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="S20" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="S20" s="1" t="s">
+      <c r="T20" s="1" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="21" spans="1:19" ht="13">
+    <row r="21" spans="1:20" ht="13">
       <c r="A21" s="1" t="s">
         <v>138</v>
       </c>
@@ -1493,28 +1557,31 @@
         <v>19</v>
       </c>
       <c r="C21" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D21" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="E21" s="1">
+      <c r="F21" s="1">
         <v>7</v>
       </c>
-      <c r="G21" s="5">
+      <c r="H21" s="5">
         <v>4810</v>
       </c>
-      <c r="O21" s="5">
+      <c r="P21" s="5">
         <v>4810</v>
-      </c>
-      <c r="P21" s="1" t="s">
-        <v>99</v>
       </c>
       <c r="Q21" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="S21" s="1" t="s">
+      <c r="R21" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="T21" s="1" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="22" spans="1:19" ht="13">
+    <row r="22" spans="1:20" ht="13">
       <c r="A22" s="1" t="s">
         <v>138</v>
       </c>
@@ -1522,34 +1589,37 @@
         <v>20</v>
       </c>
       <c r="C22" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="E22" s="1">
+      <c r="F22" s="1">
         <v>0</v>
       </c>
-      <c r="G22" s="5">
+      <c r="H22" s="5">
         <v>5495</v>
       </c>
-      <c r="L22" s="7"/>
       <c r="M22" s="7"/>
       <c r="N22" s="7"/>
-      <c r="O22" s="5">
+      <c r="O22" s="7"/>
+      <c r="P22" s="5">
         <v>5495</v>
-      </c>
-      <c r="P22" s="1" t="s">
-        <v>106</v>
       </c>
       <c r="Q22" s="1" t="s">
         <v>106</v>
       </c>
       <c r="R22" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="S22" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="S22" s="1" t="s">
+      <c r="T22" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="23" spans="1:19" ht="13">
+    <row r="23" spans="1:20" ht="13">
       <c r="A23" s="1" t="s">
         <v>138</v>
       </c>
@@ -1557,28 +1627,31 @@
         <v>21</v>
       </c>
       <c r="C23" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D23" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="E23" s="1">
+      <c r="F23" s="1">
         <v>0</v>
       </c>
-      <c r="G23" s="5">
+      <c r="H23" s="5">
         <v>5206</v>
       </c>
-      <c r="O23" s="5">
+      <c r="P23" s="5">
         <v>5206</v>
-      </c>
-      <c r="P23" s="1" t="s">
-        <v>106</v>
       </c>
       <c r="Q23" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="S23" s="1" t="s">
+      <c r="R23" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="T23" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="24" spans="1:19" ht="13">
+    <row r="24" spans="1:20" ht="13">
       <c r="A24" s="1" t="s">
         <v>138</v>
       </c>
@@ -1586,31 +1659,34 @@
         <v>22</v>
       </c>
       <c r="C24" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D24" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="E24" s="1">
-        <v>30</v>
-      </c>
-      <c r="G24" s="5">
+      <c r="F24" s="1">
+        <v>30</v>
+      </c>
+      <c r="H24" s="5">
         <v>21699.96</v>
       </c>
-      <c r="O24" s="5">
+      <c r="P24" s="5">
         <v>21699.96</v>
       </c>
-      <c r="P24" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="Q24" s="1" t="s">
         <v>97</v>
       </c>
       <c r="R24" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="S24" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="S24" s="1" t="s">
+      <c r="T24" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="25" spans="1:19" ht="13">
+    <row r="25" spans="1:20" ht="13">
       <c r="A25" s="1" t="s">
         <v>138</v>
       </c>
@@ -1618,35 +1694,38 @@
         <v>23</v>
       </c>
       <c r="C25" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D25" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="D25" s="2"/>
-      <c r="E25" s="1">
-        <v>30</v>
-      </c>
-      <c r="G25" s="5">
+      <c r="E25" s="2"/>
+      <c r="F25" s="1">
+        <v>30</v>
+      </c>
+      <c r="H25" s="5">
         <v>7355.44</v>
       </c>
-      <c r="L25" s="7"/>
       <c r="M25" s="7"/>
       <c r="N25" s="7"/>
-      <c r="O25" s="5">
+      <c r="O25" s="7"/>
+      <c r="P25" s="5">
         <v>7355.44</v>
       </c>
-      <c r="P25" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="Q25" s="1" t="s">
         <v>97</v>
       </c>
       <c r="R25" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="S25" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="S25" s="1" t="s">
+      <c r="T25" s="1" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="26" spans="1:19" ht="13">
+    <row r="26" spans="1:20" ht="13">
       <c r="A26" s="1" t="s">
         <v>138</v>
       </c>
@@ -1654,28 +1733,31 @@
         <v>24</v>
       </c>
       <c r="C26" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D26" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="E26" s="1">
-        <v>30</v>
-      </c>
-      <c r="G26" s="5">
+      <c r="F26" s="1">
+        <v>30</v>
+      </c>
+      <c r="H26" s="5">
         <v>5030.6400000000003</v>
       </c>
-      <c r="O26" s="5">
+      <c r="P26" s="5">
         <v>5030.6400000000003</v>
       </c>
-      <c r="P26" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="Q26" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="S26" s="1" t="s">
+      <c r="R26" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="T26" s="1" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="27" spans="1:19" ht="13">
+    <row r="27" spans="1:20" ht="13">
       <c r="A27" s="1" t="s">
         <v>138</v>
       </c>
@@ -1683,24 +1765,27 @@
         <v>93</v>
       </c>
       <c r="C27" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="D27" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="E27" s="1">
-        <v>30</v>
-      </c>
-      <c r="H27" s="6"/>
-      <c r="O27" s="5"/>
-      <c r="P27" s="1" t="s">
-        <v>97</v>
-      </c>
+      <c r="F27" s="1">
+        <v>30</v>
+      </c>
+      <c r="I27" s="6"/>
+      <c r="P27" s="5"/>
       <c r="Q27" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="S27" s="1" t="s">
+      <c r="R27" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="T27" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="28" spans="1:19" ht="13">
+    <row r="28" spans="1:20" ht="13">
       <c r="A28" s="1" t="s">
         <v>138</v>
       </c>
@@ -1708,31 +1793,34 @@
         <v>25</v>
       </c>
       <c r="C28" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D28" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="E28" s="1">
-        <v>30</v>
-      </c>
-      <c r="G28" s="5">
+      <c r="F28" s="1">
+        <v>30</v>
+      </c>
+      <c r="H28" s="5">
         <v>6325</v>
       </c>
-      <c r="O28" s="5">
+      <c r="P28" s="5">
         <v>6325</v>
       </c>
-      <c r="P28" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="Q28" s="1" t="s">
         <v>97</v>
       </c>
       <c r="R28" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="S28" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="S28" s="1" t="s">
+      <c r="T28" s="1" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="29" spans="1:19" ht="13">
+    <row r="29" spans="1:20" ht="13">
       <c r="A29" s="1" t="s">
         <v>138</v>
       </c>
@@ -1740,29 +1828,32 @@
         <v>26</v>
       </c>
       <c r="C29" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D29" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="E29" s="1">
-        <v>30</v>
-      </c>
-      <c r="G29" s="5">
+      <c r="F29" s="1">
+        <v>30</v>
+      </c>
+      <c r="H29" s="5">
         <v>24150</v>
       </c>
-      <c r="H29" s="6"/>
-      <c r="O29" s="5">
+      <c r="I29" s="6"/>
+      <c r="P29" s="5">
         <v>24150</v>
       </c>
-      <c r="P29" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="Q29" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="S29" s="1" t="s">
+      <c r="R29" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="T29" s="1" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="30" spans="1:19" ht="13">
+    <row r="30" spans="1:20" ht="13">
       <c r="A30" s="1" t="s">
         <v>138</v>
       </c>
@@ -1770,34 +1861,37 @@
         <v>27</v>
       </c>
       <c r="C30" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D30" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="E30" s="1">
+      <c r="F30" s="1">
         <v>0</v>
       </c>
-      <c r="G30" s="5">
+      <c r="H30" s="5">
         <v>37986.800000000003</v>
       </c>
-      <c r="L30" s="7"/>
       <c r="M30" s="7"/>
       <c r="N30" s="7"/>
-      <c r="O30" s="5">
+      <c r="O30" s="7"/>
+      <c r="P30" s="5">
         <v>37986.800000000003</v>
-      </c>
-      <c r="P30" s="1" t="s">
-        <v>106</v>
       </c>
       <c r="Q30" s="1" t="s">
         <v>106</v>
       </c>
       <c r="R30" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="S30" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="S30" s="1" t="s">
+      <c r="T30" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="31" spans="1:19" ht="13">
+    <row r="31" spans="1:20" ht="13">
       <c r="A31" s="1" t="s">
         <v>138</v>
       </c>
@@ -1805,28 +1899,31 @@
         <v>28</v>
       </c>
       <c r="C31" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D31" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="E31" s="1">
+      <c r="F31" s="1">
         <v>0</v>
       </c>
-      <c r="G31" s="5">
+      <c r="H31" s="5">
         <v>6963.41</v>
       </c>
-      <c r="O31" s="5">
+      <c r="P31" s="5">
         <v>6963.41</v>
-      </c>
-      <c r="P31" s="1" t="s">
-        <v>124</v>
       </c>
       <c r="Q31" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="S31" s="1" t="s">
+      <c r="R31" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="T31" s="1" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="32" spans="1:19" ht="13">
+    <row r="32" spans="1:20" ht="13">
       <c r="A32" s="1" t="s">
         <v>138</v>
       </c>
@@ -1834,28 +1931,31 @@
         <v>29</v>
       </c>
       <c r="C32" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D32" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="E32" s="1">
+      <c r="F32" s="1">
         <v>0</v>
       </c>
-      <c r="G32" s="5">
+      <c r="H32" s="5">
         <v>6863.01</v>
       </c>
-      <c r="O32" s="5">
+      <c r="P32" s="5">
         <v>6863.01</v>
-      </c>
-      <c r="P32" s="1" t="s">
-        <v>106</v>
       </c>
       <c r="Q32" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="S32" s="1" t="s">
+      <c r="R32" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="T32" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="33" spans="1:19" ht="13">
+    <row r="33" spans="1:20" ht="13">
       <c r="A33" s="1" t="s">
         <v>138</v>
       </c>
@@ -1863,23 +1963,26 @@
         <v>30</v>
       </c>
       <c r="C33" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D33" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="E33" s="1">
-        <v>30</v>
-      </c>
-      <c r="O33" s="5"/>
-      <c r="P33" s="1" t="s">
-        <v>97</v>
-      </c>
+      <c r="F33" s="1">
+        <v>30</v>
+      </c>
+      <c r="P33" s="5"/>
       <c r="Q33" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="S33" s="1" t="s">
+      <c r="R33" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="T33" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="34" spans="1:19" ht="13">
+    <row r="34" spans="1:20" ht="13">
       <c r="A34" s="1" t="s">
         <v>138</v>
       </c>
@@ -1887,32 +1990,35 @@
         <v>31</v>
       </c>
       <c r="C34" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D34" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="E34" s="1">
-        <v>30</v>
-      </c>
-      <c r="G34" s="5">
+      <c r="F34" s="1">
+        <v>30</v>
+      </c>
+      <c r="H34" s="5">
         <v>6367.36</v>
       </c>
-      <c r="H34" s="6"/>
-      <c r="O34" s="5">
+      <c r="I34" s="6"/>
+      <c r="P34" s="5">
         <v>6367.36</v>
       </c>
-      <c r="P34" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="Q34" s="1" t="s">
         <v>97</v>
       </c>
       <c r="R34" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="S34" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="S34" s="1" t="s">
+      <c r="T34" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="35" spans="1:19" ht="13">
+    <row r="35" spans="1:20" ht="13">
       <c r="A35" s="1" t="s">
         <v>138</v>
       </c>
@@ -1920,34 +2026,37 @@
         <v>32</v>
       </c>
       <c r="C35" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D35" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="E35" s="1">
+      <c r="F35" s="1">
         <v>0</v>
       </c>
-      <c r="G35" s="5">
+      <c r="H35" s="5">
         <v>5116.7</v>
       </c>
-      <c r="L35" s="7"/>
       <c r="M35" s="7"/>
       <c r="N35" s="7"/>
-      <c r="O35" s="5">
+      <c r="O35" s="7"/>
+      <c r="P35" s="5">
         <v>5116.7</v>
-      </c>
-      <c r="P35" s="1" t="s">
-        <v>106</v>
       </c>
       <c r="Q35" s="1" t="s">
         <v>106</v>
       </c>
       <c r="R35" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="S35" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="S35" s="1" t="s">
+      <c r="T35" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="36" spans="1:19" ht="13">
+    <row r="36" spans="1:20" ht="13">
       <c r="A36" s="1" t="s">
         <v>138</v>
       </c>
@@ -1955,31 +2064,34 @@
         <v>33</v>
       </c>
       <c r="C36" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D36" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="E36" s="1">
+      <c r="F36" s="1">
         <v>7</v>
       </c>
-      <c r="G36" s="5">
+      <c r="H36" s="5">
         <v>4743.3100000000004</v>
       </c>
-      <c r="O36" s="5">
+      <c r="P36" s="5">
         <v>4743.3100000000004</v>
-      </c>
-      <c r="P36" s="1" t="s">
-        <v>99</v>
       </c>
       <c r="Q36" s="1" t="s">
         <v>99</v>
       </c>
       <c r="R36" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="S36" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="S36" s="1" t="s">
+      <c r="T36" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="37" spans="1:19" ht="13">
+    <row r="37" spans="1:20" ht="13">
       <c r="A37" s="1" t="s">
         <v>138</v>
       </c>
@@ -1987,28 +2099,31 @@
         <v>34</v>
       </c>
       <c r="C37" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D37" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="E37" s="1">
+      <c r="F37" s="1">
         <v>0</v>
       </c>
-      <c r="G37" s="5">
+      <c r="H37" s="5">
         <v>193540.4</v>
       </c>
-      <c r="O37" s="5">
+      <c r="P37" s="5">
         <v>193540.4</v>
       </c>
-      <c r="P37" s="1" t="s">
+      <c r="Q37" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="Q37" s="1">
+      <c r="R37" s="1">
         <v>0</v>
       </c>
-      <c r="S37" s="1" t="s">
+      <c r="T37" s="1" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="38" spans="1:19" ht="13">
+    <row r="38" spans="1:20" ht="13">
       <c r="A38" s="1" t="s">
         <v>138</v>
       </c>
@@ -2016,29 +2131,32 @@
         <v>35</v>
       </c>
       <c r="C38" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D38" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="D38" s="2"/>
-      <c r="E38" s="1">
-        <v>30</v>
-      </c>
-      <c r="G38" s="5">
+      <c r="E38" s="2"/>
+      <c r="F38" s="1">
+        <v>30</v>
+      </c>
+      <c r="H38" s="5">
         <v>6325</v>
       </c>
-      <c r="O38" s="5">
+      <c r="P38" s="5">
         <v>6325</v>
       </c>
-      <c r="P38" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="Q38" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="S38" s="1" t="s">
+      <c r="R38" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="T38" s="1" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="39" spans="1:19" ht="13">
+    <row r="39" spans="1:20" ht="13">
       <c r="A39" s="1" t="s">
         <v>138</v>
       </c>
@@ -2046,23 +2164,26 @@
         <v>36</v>
       </c>
       <c r="C39" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D39" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="D39" s="2"/>
-      <c r="G39" s="5">
+      <c r="E39" s="2"/>
+      <c r="H39" s="5">
         <v>30395.82</v>
       </c>
-      <c r="O39" s="5">
+      <c r="P39" s="5">
         <v>30395.82</v>
       </c>
-      <c r="P39" s="1" t="s">
+      <c r="Q39" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="S39" s="1" t="s">
+      <c r="T39" s="1" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="40" spans="1:19" ht="13">
+    <row r="40" spans="1:20" ht="13">
       <c r="A40" s="1" t="s">
         <v>138</v>
       </c>
@@ -2070,23 +2191,26 @@
         <v>37</v>
       </c>
       <c r="C40" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D40" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="E40" s="1">
+      <c r="F40" s="1">
         <v>7</v>
       </c>
-      <c r="O40" s="5"/>
-      <c r="P40" s="1" t="s">
-        <v>99</v>
-      </c>
+      <c r="P40" s="5"/>
       <c r="Q40" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="S40" s="1" t="s">
+      <c r="R40" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="T40" s="1" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="41" spans="1:19" ht="13">
+    <row r="41" spans="1:20" ht="13">
       <c r="A41" s="1" t="s">
         <v>138</v>
       </c>
@@ -2094,28 +2218,31 @@
         <v>38</v>
       </c>
       <c r="C41" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D41" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="E41" s="1">
-        <v>30</v>
-      </c>
-      <c r="G41" s="5">
+      <c r="F41" s="1">
+        <v>30</v>
+      </c>
+      <c r="H41" s="5">
         <v>8301.2099999999991</v>
       </c>
-      <c r="O41" s="5">
+      <c r="P41" s="5">
         <v>8301.2099999999991</v>
       </c>
-      <c r="P41" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="Q41" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="S41" s="1" t="s">
+      <c r="R41" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="T41" s="1" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="42" spans="1:19" ht="13">
+    <row r="42" spans="1:20" ht="13">
       <c r="A42" s="1" t="s">
         <v>138</v>
       </c>
@@ -2123,28 +2250,31 @@
         <v>39</v>
       </c>
       <c r="C42" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D42" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="E42" s="1">
-        <v>30</v>
-      </c>
-      <c r="G42" s="5">
+      <c r="F42" s="1">
+        <v>30</v>
+      </c>
+      <c r="H42" s="5">
         <v>40919.9</v>
       </c>
-      <c r="O42" s="5">
+      <c r="P42" s="5">
         <v>40919.9</v>
       </c>
-      <c r="P42" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="Q42" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="S42" s="1" t="s">
+      <c r="R42" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="T42" s="1" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="43" spans="1:19" ht="13">
+    <row r="43" spans="1:20" ht="13">
       <c r="A43" s="1" t="s">
         <v>138</v>
       </c>
@@ -2152,26 +2282,29 @@
         <v>40</v>
       </c>
       <c r="C43" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D43" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="E43" s="1">
-        <v>30</v>
-      </c>
-      <c r="O43" s="5"/>
-      <c r="P43" s="1" t="s">
-        <v>97</v>
-      </c>
+      <c r="F43" s="1">
+        <v>30</v>
+      </c>
+      <c r="P43" s="5"/>
       <c r="Q43" s="1" t="s">
         <v>97</v>
       </c>
       <c r="R43" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="S43" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="S43" s="1" t="s">
+      <c r="T43" s="1" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="44" spans="1:19" ht="13">
+    <row r="44" spans="1:20" ht="13">
       <c r="A44" s="1" t="s">
         <v>138</v>
       </c>
@@ -2179,31 +2312,34 @@
         <v>41</v>
       </c>
       <c r="C44" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D44" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="E44" s="1">
-        <v>30</v>
-      </c>
-      <c r="G44" s="5">
+      <c r="F44" s="1">
+        <v>30</v>
+      </c>
+      <c r="H44" s="5">
         <v>7116</v>
       </c>
-      <c r="O44" s="5">
+      <c r="P44" s="5">
         <v>7116</v>
       </c>
-      <c r="P44" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="Q44" s="1" t="s">
         <v>97</v>
       </c>
       <c r="R44" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="S44" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="S44" s="3" t="s">
+      <c r="T44" s="3" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="45" spans="1:19" ht="13">
+    <row r="45" spans="1:20" ht="13">
       <c r="A45" s="1" t="s">
         <v>138</v>
       </c>
@@ -2211,28 +2347,31 @@
         <v>42</v>
       </c>
       <c r="C45" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D45" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="E45" s="1">
+      <c r="F45" s="1">
         <v>0</v>
       </c>
-      <c r="G45" s="5">
+      <c r="H45" s="5">
         <v>6469.35</v>
       </c>
-      <c r="O45" s="5">
+      <c r="P45" s="5">
         <v>6469.35</v>
-      </c>
-      <c r="P45" s="1" t="s">
-        <v>106</v>
       </c>
       <c r="Q45" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="S45" s="1" t="s">
+      <c r="R45" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="T45" s="1" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="46" spans="1:19" ht="13">
+    <row r="46" spans="1:20" ht="13">
       <c r="A46" s="1" t="s">
         <v>138</v>
       </c>
@@ -2240,29 +2379,32 @@
         <v>43</v>
       </c>
       <c r="C46" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D46" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="D46" s="2"/>
-      <c r="E46" s="1">
+      <c r="E46" s="2"/>
+      <c r="F46" s="1">
         <v>0</v>
       </c>
-      <c r="G46" s="5">
+      <c r="H46" s="5">
         <v>5227.2</v>
       </c>
-      <c r="O46" s="5">
+      <c r="P46" s="5">
         <v>5227.2</v>
-      </c>
-      <c r="P46" s="1" t="s">
-        <v>106</v>
       </c>
       <c r="Q46" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="S46" s="1" t="s">
+      <c r="R46" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="T46" s="1" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="47" spans="1:19" ht="13">
+    <row r="47" spans="1:20" ht="13">
       <c r="A47" s="1" t="s">
         <v>138</v>
       </c>
@@ -2270,19 +2412,22 @@
         <v>44</v>
       </c>
       <c r="C47" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D47" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="G47" s="5">
+      <c r="H47" s="5">
         <v>9348</v>
       </c>
-      <c r="O47" s="5">
+      <c r="P47" s="5">
         <v>9348</v>
       </c>
-      <c r="S47" s="1" t="s">
+      <c r="T47" s="1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="48" spans="1:19" ht="13">
+    <row r="48" spans="1:20" ht="13">
       <c r="A48" s="1" t="s">
         <v>138</v>
       </c>
@@ -2290,29 +2435,32 @@
         <v>45</v>
       </c>
       <c r="C48" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D48" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="D48" s="2"/>
-      <c r="E48" s="1">
+      <c r="E48" s="2"/>
+      <c r="F48" s="1">
         <v>0</v>
       </c>
-      <c r="G48" s="5">
+      <c r="H48" s="5">
         <v>8202</v>
       </c>
-      <c r="O48" s="5">
+      <c r="P48" s="5">
         <v>8202</v>
-      </c>
-      <c r="P48" s="1" t="s">
-        <v>106</v>
       </c>
       <c r="Q48" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="S48" s="1" t="s">
+      <c r="R48" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="T48" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="49" spans="1:19" ht="13">
+    <row r="49" spans="1:20" ht="13">
       <c r="A49" s="1" t="s">
         <v>138</v>
       </c>
@@ -2320,31 +2468,34 @@
         <v>46</v>
       </c>
       <c r="C49" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D49" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="E49" s="1">
+      <c r="F49" s="1">
         <v>0</v>
       </c>
-      <c r="G49" s="5">
+      <c r="H49" s="5">
         <v>8634.1</v>
       </c>
-      <c r="O49" s="5">
+      <c r="P49" s="5">
         <v>8634.1</v>
-      </c>
-      <c r="P49" s="1" t="s">
-        <v>106</v>
       </c>
       <c r="Q49" s="1" t="s">
         <v>106</v>
       </c>
       <c r="R49" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="S49" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="S49" s="1" t="s">
+      <c r="T49" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="50" spans="1:19" ht="13">
+    <row r="50" spans="1:20" ht="13">
       <c r="A50" s="1" t="s">
         <v>138</v>
       </c>
@@ -2352,28 +2503,31 @@
         <v>47</v>
       </c>
       <c r="C50" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D50" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="E50" s="1">
+      <c r="F50" s="1">
         <v>7</v>
       </c>
-      <c r="G50" s="5">
+      <c r="H50" s="5">
         <v>5131.25</v>
       </c>
-      <c r="O50" s="5">
+      <c r="P50" s="5">
         <v>5131.25</v>
-      </c>
-      <c r="P50" s="1" t="s">
-        <v>99</v>
       </c>
       <c r="Q50" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="S50" s="1" t="s">
+      <c r="R50" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="T50" s="1" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="51" spans="1:19" ht="13">
+    <row r="51" spans="1:20" ht="13">
       <c r="A51" s="1" t="s">
         <v>138</v>
       </c>
@@ -2381,27 +2535,30 @@
         <v>48</v>
       </c>
       <c r="C51" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D51" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="E51" s="1">
+      <c r="F51" s="1">
         <v>0</v>
       </c>
-      <c r="G51" s="5">
+      <c r="H51" s="5">
         <v>5495</v>
       </c>
-      <c r="O51" s="5">
+      <c r="P51" s="5">
         <v>5495</v>
-      </c>
-      <c r="P51" s="1" t="s">
-        <v>106</v>
       </c>
       <c r="Q51" s="1" t="s">
         <v>106</v>
       </c>
       <c r="R51" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="S51" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="S51" s="1" t="s">
+      <c r="T51" s="1" t="s">
         <v>151</v>
       </c>
     </row>

</xml_diff>